<commit_message>
Update testing checklist with iPads
</commit_message>
<xml_diff>
--- a/docs/testing-checklist.xlsx
+++ b/docs/testing-checklist.xlsx
@@ -591,8 +591,8 @@
       <c r="C5" s="8" t="n"/>
       <c r="D5" s="8" t="n"/>
       <c r="E5" s="8" t="n"/>
-      <c r="F5" s="4" t="n"/>
-      <c r="G5" s="4" t="n"/>
+      <c r="F5" s="8" t="n"/>
+      <c r="G5" s="8" t="n"/>
       <c r="H5" s="9" t="n"/>
     </row>
     <row r="6">
@@ -637,8 +637,8 @@
       <c r="C8" s="8" t="n"/>
       <c r="D8" s="8" t="n"/>
       <c r="E8" s="8" t="n"/>
-      <c r="F8" s="4" t="n"/>
-      <c r="G8" s="4" t="n"/>
+      <c r="F8" s="8" t="n"/>
+      <c r="G8" s="8" t="n"/>
       <c r="H8" s="15" t="n"/>
     </row>
     <row r="9">
@@ -725,8 +725,8 @@
       <c r="C14" s="8" t="n"/>
       <c r="D14" s="8" t="n"/>
       <c r="E14" s="8" t="n"/>
-      <c r="F14" s="4" t="n"/>
-      <c r="G14" s="4" t="n"/>
+      <c r="F14" s="8" t="n"/>
+      <c r="G14" s="8" t="n"/>
       <c r="H14" s="9" t="n"/>
     </row>
     <row r="15">
@@ -813,8 +813,8 @@
       <c r="C20" s="8" t="n"/>
       <c r="D20" s="8" t="n"/>
       <c r="E20" s="8" t="n"/>
-      <c r="F20" s="4" t="n"/>
-      <c r="G20" s="4" t="n"/>
+      <c r="F20" s="8" t="n"/>
+      <c r="G20" s="8" t="n"/>
       <c r="H20" s="15" t="n"/>
     </row>
     <row r="21">
@@ -901,8 +901,8 @@
       <c r="C26" s="8" t="n"/>
       <c r="D26" s="8" t="n"/>
       <c r="E26" s="8" t="n"/>
-      <c r="F26" s="4" t="n"/>
-      <c r="G26" s="4" t="n"/>
+      <c r="F26" s="8" t="n"/>
+      <c r="G26" s="8" t="n"/>
       <c r="H26" s="9" t="n"/>
     </row>
     <row r="27">
@@ -989,8 +989,8 @@
       <c r="C32" s="8" t="n"/>
       <c r="D32" s="8" t="n"/>
       <c r="E32" s="8" t="n"/>
-      <c r="F32" s="4" t="n"/>
-      <c r="G32" s="4" t="n"/>
+      <c r="F32" s="8" t="n"/>
+      <c r="G32" s="8" t="n"/>
       <c r="H32" s="15" t="n"/>
     </row>
     <row r="33">
@@ -1077,8 +1077,8 @@
       <c r="C38" s="8" t="n"/>
       <c r="D38" s="8" t="n"/>
       <c r="E38" s="8" t="n"/>
-      <c r="F38" s="4" t="n"/>
-      <c r="G38" s="4" t="n"/>
+      <c r="F38" s="8" t="n"/>
+      <c r="G38" s="8" t="n"/>
       <c r="H38" s="9" t="n"/>
     </row>
     <row r="39">
@@ -1109,8 +1109,8 @@
       <c r="C40" s="8" t="n"/>
       <c r="D40" s="8" t="n"/>
       <c r="E40" s="8" t="n"/>
-      <c r="F40" s="4" t="n"/>
-      <c r="G40" s="4" t="n"/>
+      <c r="F40" s="8" t="n"/>
+      <c r="G40" s="8" t="n"/>
       <c r="H40" s="15" t="n"/>
     </row>
     <row r="41">
@@ -1155,8 +1155,8 @@
       <c r="C43" s="8" t="n"/>
       <c r="D43" s="8" t="n"/>
       <c r="E43" s="8" t="n"/>
-      <c r="F43" s="4" t="n"/>
-      <c r="G43" s="4" t="n"/>
+      <c r="F43" s="8" t="n"/>
+      <c r="G43" s="8" t="n"/>
       <c r="H43" s="9" t="n"/>
     </row>
     <row r="44">
@@ -1215,8 +1215,8 @@
       <c r="C47" s="8" t="n"/>
       <c r="D47" s="8" t="n"/>
       <c r="E47" s="8" t="n"/>
-      <c r="F47" s="4" t="n"/>
-      <c r="G47" s="4" t="n"/>
+      <c r="F47" s="8" t="n"/>
+      <c r="G47" s="8" t="n"/>
       <c r="H47" s="15" t="n"/>
     </row>
     <row r="48">
@@ -1275,8 +1275,8 @@
       <c r="C51" s="8" t="n"/>
       <c r="D51" s="8" t="n"/>
       <c r="E51" s="8" t="n"/>
-      <c r="F51" s="4" t="n"/>
-      <c r="G51" s="4" t="n"/>
+      <c r="F51" s="8" t="n"/>
+      <c r="G51" s="8" t="n"/>
       <c r="H51" s="9" t="n"/>
     </row>
     <row r="52">
@@ -1321,8 +1321,8 @@
       <c r="C54" s="8" t="n"/>
       <c r="D54" s="8" t="n"/>
       <c r="E54" s="8" t="n"/>
-      <c r="F54" s="4" t="n"/>
-      <c r="G54" s="4" t="n"/>
+      <c r="F54" s="8" t="n"/>
+      <c r="G54" s="8" t="n"/>
       <c r="H54" s="15" t="n"/>
     </row>
     <row r="55">
@@ -1409,8 +1409,8 @@
       <c r="C60" s="8" t="n"/>
       <c r="D60" s="8" t="n"/>
       <c r="E60" s="8" t="n"/>
-      <c r="F60" s="4" t="n"/>
-      <c r="G60" s="4" t="n"/>
+      <c r="F60" s="8" t="n"/>
+      <c r="G60" s="8" t="n"/>
       <c r="H60" s="9" t="n"/>
     </row>
     <row r="61">
@@ -1455,8 +1455,8 @@
       <c r="C63" s="8" t="n"/>
       <c r="D63" s="8" t="n"/>
       <c r="E63" s="8" t="n"/>
-      <c r="F63" s="4" t="n"/>
-      <c r="G63" s="4" t="n"/>
+      <c r="F63" s="8" t="n"/>
+      <c r="G63" s="8" t="n"/>
       <c r="H63" s="15" t="n"/>
     </row>
     <row r="64">
@@ -1487,8 +1487,8 @@
       <c r="C65" s="8" t="n"/>
       <c r="D65" s="8" t="n"/>
       <c r="E65" s="8" t="n"/>
-      <c r="F65" s="4" t="n"/>
-      <c r="G65" s="4" t="n"/>
+      <c r="F65" s="8" t="n"/>
+      <c r="G65" s="8" t="n"/>
       <c r="H65" s="9" t="n"/>
     </row>
   </sheetData>

</xml_diff>